<commit_message>
Fix issues from testing
- finalize_draft.py --no-etag strips //_ keys from the BMKB draft;
  validate_bmkb.py points to it.
- censor_state_for_reported() resolves results as reported ('<0.006');
  the converter uses it to check bounded results too.
- Naming rule for tBCO/rBCO object ids and run ids; gold rBCO ids and
  xlsx RBCOID cells renamed and re-finalized.
- Preflight reports condition.id and condition.name separately.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/troponin_I/Troponin_I_SDTM.xlsx
+++ b/examples/troponin_I/Troponin_I_SDTM.xlsx
@@ -703,7 +703,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -846,7 +845,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
@@ -854,7 +852,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
@@ -984,7 +981,6 @@
       <c r="H18" s="14" t="n"/>
       <c r="I18" s="12" t="n"/>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
@@ -6093,6 +6089,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -6287,7 +6284,7 @@
       </c>
       <c r="H6" s="31" t="inlineStr">
         <is>
-          <t>https://biocomputeobject.org/PLACEHOLDER_Troponin_I_patient1_rBCO/1.0.0</t>
+          <t>https://biocomputeobject.org/PLACEHOLDER_Troponin_I_BM-2026-01-001_R-2026-0315-01_rBCO/1.0.0</t>
         </is>
       </c>
       <c r="I6" s="31" t="inlineStr">
@@ -6593,7 +6590,7 @@
       </c>
       <c r="H12" s="31" t="inlineStr">
         <is>
-          <t>https://biocomputeobject.org/PLACEHOLDER_Troponin_I_patient2_rBCO/1.0.0</t>
+          <t>https://biocomputeobject.org/PLACEHOLDER_Troponin_I_BM-2026-01-002_R-2026-0316-01_rBCO/1.0.0</t>
         </is>
       </c>
       <c r="I12" s="31" t="inlineStr">

</xml_diff>

<commit_message>
Apply T03, T04, T05, T07; correct AMI to DOID:9408
- scripts/ols_lookup.py: OLS4 web API lookup (adapted from
  ontology_mapper/src/ols.py), ranking by exact label, resource order and
  species; `get` to verify a CURIE.
- references/cdisc-ct/ extract (NCI EVS 2026-09-25) + scripts/cdisc_ct.py
  with synonym resolution; converter prints CT notes.
- SKILL.md: document precedence rule, CT and OLS lookup steps.
- Gold tBCO filled only from the fixtures; acute myocardial infarction is
  DOID:9408 (DOID:5844 is myocardial infarction) across gold and docs.

run_checks.py: 9/9 self-tests, 346/346 gold cells.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/troponin_I/Troponin_I_SDTM.xlsx
+++ b/examples/troponin_I/Troponin_I_SDTM.xlsx
@@ -703,6 +703,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -845,6 +846,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
@@ -852,6 +854,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
@@ -981,6 +984,7 @@
       <c r="H18" s="14" t="n"/>
       <c r="I18" s="12" t="n"/>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
@@ -4762,6 +4766,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -5018,6 +5023,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -6803,6 +6809,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -7120,7 +7127,7 @@
       </c>
       <c r="K5" s="31" t="inlineStr">
         <is>
-          <t>DOID:5844</t>
+          <t>DOID:9408</t>
         </is>
       </c>
       <c r="L5" s="31" t="inlineStr">
@@ -7252,7 +7259,7 @@
       </c>
       <c r="K6" s="31" t="inlineStr">
         <is>
-          <t>DOID:5844</t>
+          <t>DOID:9408</t>
         </is>
       </c>
       <c r="L6" s="31" t="inlineStr">

</xml_diff>